<commit_message>
updated data exportation functionality, updated in main.py
</commit_message>
<xml_diff>
--- a/data/output/output_data.xlsx
+++ b/data/output/output_data.xlsx
@@ -1,3 +1,20 @@
+
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet name="1001" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="1004" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2004" sheetId="3" state="visible" r:id="rId3"/>
+  </sheets>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+</workbook>
+</file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
@@ -390,4 +407,1462 @@
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
 </a:theme>
+</file>
+
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Z-Score Percentile</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>z_score</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>z_score_deviation (%)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>anomaly</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>0.9078412990032004</v>
+      </c>
+      <c r="B4" t="n">
+        <v>81.80189624487603</v>
+      </c>
+      <c r="C4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>-0.4458689170643704</v>
+      </c>
+      <c r="B5" t="n">
+        <v>32.78459680434778</v>
+      </c>
+      <c r="C5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>-0.8925123611712381</v>
+      </c>
+      <c r="B6" t="n">
+        <v>18.60591850893152</v>
+      </c>
+      <c r="C6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>-0.7487728481926048</v>
+      </c>
+      <c r="B7" t="n">
+        <v>22.69970637366298</v>
+      </c>
+      <c r="C7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>-0.8969096265694753</v>
+      </c>
+      <c r="B8" t="n">
+        <v>18.4883571432826</v>
+      </c>
+      <c r="C8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>-0.8969037057031658</v>
+      </c>
+      <c r="B9" t="n">
+        <v>18.48851512726382</v>
+      </c>
+      <c r="C9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>-0.7487734683146702</v>
+      </c>
+      <c r="B10" t="n">
+        <v>22.69968768228979</v>
+      </c>
+      <c r="C10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>0.5915925417082991</v>
+      </c>
+      <c r="B11" t="n">
+        <v>72.29382653025299</v>
+      </c>
+      <c r="C11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>-1.324557654660229</v>
+      </c>
+      <c r="B12" t="n">
+        <v>9.265895429722764</v>
+      </c>
+      <c r="C12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>-0.2270710655802821</v>
+      </c>
+      <c r="B13" t="n">
+        <v>41.01842413639275</v>
+      </c>
+      <c r="C13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>-0.7134764738416087</v>
+      </c>
+      <c r="B14" t="n">
+        <v>23.77754830025104</v>
+      </c>
+      <c r="C14" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>-0.7410039273935294</v>
+      </c>
+      <c r="B15" t="n">
+        <v>22.93455295125452</v>
+      </c>
+      <c r="C15" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>0.2589370049199478</v>
+      </c>
+      <c r="B16" t="n">
+        <v>60.21580770950496</v>
+      </c>
+      <c r="C16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>-0.3541441234874145</v>
+      </c>
+      <c r="B17" t="n">
+        <v>36.16154381406916</v>
+      </c>
+      <c r="C17" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>-0.5039287831891985</v>
+      </c>
+      <c r="B18" t="n">
+        <v>30.71557116144048</v>
+      </c>
+      <c r="C18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>-0.365358003149192</v>
+      </c>
+      <c r="B19" t="n">
+        <v>35.74220930849559</v>
+      </c>
+      <c r="C19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>-0.3748926157689837</v>
+      </c>
+      <c r="B20" t="n">
+        <v>35.38701655045149</v>
+      </c>
+      <c r="C20" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>-0.7494193580132499</v>
+      </c>
+      <c r="B21" t="n">
+        <v>22.68022434820888</v>
+      </c>
+      <c r="C21" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Payroll Rule Results</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Anomaly</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PF</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>8991</v>
+      </c>
+      <c r="C26" t="n">
+        <v>8991</v>
+      </c>
+      <c r="D26" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>HRA</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0.5000066733400067</v>
+      </c>
+      <c r="C27" t="n">
+        <v>4.117726550623146e-06</v>
+      </c>
+      <c r="D27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Net_Payable</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>206378</v>
+      </c>
+      <c r="C28" t="n">
+        <v>330541</v>
+      </c>
+      <c r="D28" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Unsupervised Machine Learning Results</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Latest Record Anomaly? (Y/N)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Isolation Forest</t>
+        </is>
+      </c>
+      <c r="B33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Isolation Forest (Reduced)</t>
+        </is>
+      </c>
+      <c r="B34" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Local Outlier Factor</t>
+        </is>
+      </c>
+      <c r="B35" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>PCA</t>
+        </is>
+      </c>
+      <c r="B36" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Ensemble ML Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>PCA_Anomaly</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>IsolationForest_Anomaly</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>IsolationForest_Reduced_Anomaly</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LOF_Anomaly</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Ensemble_Anomaly</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>1001</v>
+      </c>
+      <c r="B41" t="b">
+        <v>0</v>
+      </c>
+      <c r="C41" t="b">
+        <v>0</v>
+      </c>
+      <c r="D41" t="b">
+        <v>0</v>
+      </c>
+      <c r="E41" t="b">
+        <v>0</v>
+      </c>
+      <c r="F41" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Root Cause Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Root Cause Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Methods</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Max_Severity</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Detected_By_Both</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Overall Verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>No Anomaly</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Z-Score Percentile</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>z_score</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>z_score_deviation (%)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>anomaly</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>0.9078412990032004</v>
+      </c>
+      <c r="B4" t="n">
+        <v>81.80189624487603</v>
+      </c>
+      <c r="C4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>-0.4458689170643704</v>
+      </c>
+      <c r="B5" t="n">
+        <v>32.78459680434778</v>
+      </c>
+      <c r="C5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>-0.8925123611712381</v>
+      </c>
+      <c r="B6" t="n">
+        <v>18.60591850893152</v>
+      </c>
+      <c r="C6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>-0.7487728481926048</v>
+      </c>
+      <c r="B7" t="n">
+        <v>22.69970637366298</v>
+      </c>
+      <c r="C7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>-0.8969096265694753</v>
+      </c>
+      <c r="B8" t="n">
+        <v>18.4883571432826</v>
+      </c>
+      <c r="C8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>-0.8969037057031658</v>
+      </c>
+      <c r="B9" t="n">
+        <v>18.48851512726382</v>
+      </c>
+      <c r="C9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>-0.7487734683146702</v>
+      </c>
+      <c r="B10" t="n">
+        <v>22.69968768228979</v>
+      </c>
+      <c r="C10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>0.5915925417082991</v>
+      </c>
+      <c r="B11" t="n">
+        <v>72.29382653025299</v>
+      </c>
+      <c r="C11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>-1.324557654660229</v>
+      </c>
+      <c r="B12" t="n">
+        <v>9.265895429722764</v>
+      </c>
+      <c r="C12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>-0.2270710655802821</v>
+      </c>
+      <c r="B13" t="n">
+        <v>41.01842413639275</v>
+      </c>
+      <c r="C13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>-0.7134764738416087</v>
+      </c>
+      <c r="B14" t="n">
+        <v>23.77754830025104</v>
+      </c>
+      <c r="C14" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>-0.7410039273935294</v>
+      </c>
+      <c r="B15" t="n">
+        <v>22.93455295125452</v>
+      </c>
+      <c r="C15" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>0.2589370049199478</v>
+      </c>
+      <c r="B16" t="n">
+        <v>60.21580770950496</v>
+      </c>
+      <c r="C16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>-0.3541441234874145</v>
+      </c>
+      <c r="B17" t="n">
+        <v>36.16154381406916</v>
+      </c>
+      <c r="C17" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>-0.5039287831891985</v>
+      </c>
+      <c r="B18" t="n">
+        <v>30.71557116144048</v>
+      </c>
+      <c r="C18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>-0.365358003149192</v>
+      </c>
+      <c r="B19" t="n">
+        <v>35.74220930849559</v>
+      </c>
+      <c r="C19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>-0.3748926157689837</v>
+      </c>
+      <c r="B20" t="n">
+        <v>35.38701655045149</v>
+      </c>
+      <c r="C20" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>-0.7494193580132499</v>
+      </c>
+      <c r="B21" t="n">
+        <v>22.68022434820888</v>
+      </c>
+      <c r="C21" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Payroll Rule Results</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Anomaly</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PF</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>8991</v>
+      </c>
+      <c r="C26" t="n">
+        <v>8991</v>
+      </c>
+      <c r="D26" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>HRA</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0.5000066733400067</v>
+      </c>
+      <c r="C27" t="n">
+        <v>4.117726550623146e-06</v>
+      </c>
+      <c r="D27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Net_Payable</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>206378</v>
+      </c>
+      <c r="C28" t="n">
+        <v>330541</v>
+      </c>
+      <c r="D28" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Unsupervised Machine Learning Results</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Latest Record Anomaly? (Y/N)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Isolation Forest</t>
+        </is>
+      </c>
+      <c r="B33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Isolation Forest (Reduced)</t>
+        </is>
+      </c>
+      <c r="B34" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Local Outlier Factor</t>
+        </is>
+      </c>
+      <c r="B35" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>PCA</t>
+        </is>
+      </c>
+      <c r="B36" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Ensemble ML Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>PCA_Anomaly</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>IsolationForest_Anomaly</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>IsolationForest_Reduced_Anomaly</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LOF_Anomaly</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Ensemble_Anomaly</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>1004</v>
+      </c>
+      <c r="B41" t="b">
+        <v>0</v>
+      </c>
+      <c r="C41" t="b">
+        <v>0</v>
+      </c>
+      <c r="D41" t="b">
+        <v>0</v>
+      </c>
+      <c r="E41" t="b">
+        <v>0</v>
+      </c>
+      <c r="F41" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Root Cause Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Root Cause Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Methods</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Max_Severity</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Detected_By_Both</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Overall Verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>No Anomaly</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Z-Score Percentile</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>z_score</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>z_score_deviation (%)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>anomaly</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>0.9078412990032004</v>
+      </c>
+      <c r="B4" t="n">
+        <v>81.80189624487603</v>
+      </c>
+      <c r="C4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>-0.4458689170643704</v>
+      </c>
+      <c r="B5" t="n">
+        <v>32.78459680434778</v>
+      </c>
+      <c r="C5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>-0.8925123611712381</v>
+      </c>
+      <c r="B6" t="n">
+        <v>18.60591850893152</v>
+      </c>
+      <c r="C6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>-0.7487728481926048</v>
+      </c>
+      <c r="B7" t="n">
+        <v>22.69970637366298</v>
+      </c>
+      <c r="C7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>-0.8969096265694753</v>
+      </c>
+      <c r="B8" t="n">
+        <v>18.4883571432826</v>
+      </c>
+      <c r="C8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>-0.8969037057031658</v>
+      </c>
+      <c r="B9" t="n">
+        <v>18.48851512726382</v>
+      </c>
+      <c r="C9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>-0.7487734683146702</v>
+      </c>
+      <c r="B10" t="n">
+        <v>22.69968768228979</v>
+      </c>
+      <c r="C10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>0.5915925417082991</v>
+      </c>
+      <c r="B11" t="n">
+        <v>72.29382653025299</v>
+      </c>
+      <c r="C11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>-1.324557654660229</v>
+      </c>
+      <c r="B12" t="n">
+        <v>9.265895429722764</v>
+      </c>
+      <c r="C12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>-0.2270710655802821</v>
+      </c>
+      <c r="B13" t="n">
+        <v>41.01842413639275</v>
+      </c>
+      <c r="C13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>-0.7134764738416087</v>
+      </c>
+      <c r="B14" t="n">
+        <v>23.77754830025104</v>
+      </c>
+      <c r="C14" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>-0.7410039273935294</v>
+      </c>
+      <c r="B15" t="n">
+        <v>22.93455295125452</v>
+      </c>
+      <c r="C15" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>0.2589370049199478</v>
+      </c>
+      <c r="B16" t="n">
+        <v>60.21580770950496</v>
+      </c>
+      <c r="C16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>-0.3541441234874145</v>
+      </c>
+      <c r="B17" t="n">
+        <v>36.16154381406916</v>
+      </c>
+      <c r="C17" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>-0.5039287831891985</v>
+      </c>
+      <c r="B18" t="n">
+        <v>30.71557116144048</v>
+      </c>
+      <c r="C18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>-0.365358003149192</v>
+      </c>
+      <c r="B19" t="n">
+        <v>35.74220930849559</v>
+      </c>
+      <c r="C19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>-0.3748926157689837</v>
+      </c>
+      <c r="B20" t="n">
+        <v>35.38701655045149</v>
+      </c>
+      <c r="C20" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>-0.7494193580132499</v>
+      </c>
+      <c r="B21" t="n">
+        <v>22.68022434820888</v>
+      </c>
+      <c r="C21" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Payroll Rule Results</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Anomaly</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PF</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>8991</v>
+      </c>
+      <c r="C26" t="n">
+        <v>8991</v>
+      </c>
+      <c r="D26" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>HRA</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0.5000066733400067</v>
+      </c>
+      <c r="C27" t="n">
+        <v>4.117726550623146e-06</v>
+      </c>
+      <c r="D27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Net_Payable</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>206378</v>
+      </c>
+      <c r="C28" t="n">
+        <v>330541</v>
+      </c>
+      <c r="D28" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Unsupervised Machine Learning Results</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Latest Record Anomaly? (Y/N)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Isolation Forest</t>
+        </is>
+      </c>
+      <c r="B33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Isolation Forest (Reduced)</t>
+        </is>
+      </c>
+      <c r="B34" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Local Outlier Factor</t>
+        </is>
+      </c>
+      <c r="B35" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>PCA</t>
+        </is>
+      </c>
+      <c r="B36" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Ensemble ML Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>PCA_Anomaly</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>IsolationForest_Anomaly</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>IsolationForest_Reduced_Anomaly</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LOF_Anomaly</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Ensemble_Anomaly</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B41" t="b">
+        <v>0</v>
+      </c>
+      <c r="C41" t="b">
+        <v>0</v>
+      </c>
+      <c r="D41" t="b">
+        <v>0</v>
+      </c>
+      <c r="E41" t="b">
+        <v>0</v>
+      </c>
+      <c r="F41" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Root Cause Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Root Cause Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Methods</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Max_Severity</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Detected_By_Both</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Overall Verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>No Anomaly</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
updated to add overall to export; updated to remove index from stats-based and make it a column
</commit_message>
<xml_diff>
--- a/data/output/output_data.xlsx
+++ b/data/output/output_data.xlsx
@@ -428,215 +428,310 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>z_score</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>z_score_deviation (%)</t>
-        </is>
-      </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>z_score_deviation</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>anomaly</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paid_days</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>0.9078412990032004</v>
       </c>
-      <c r="B4" t="n">
+      <c r="C4" t="n">
         <v>81.80189624487603</v>
       </c>
-      <c r="C4" t="b">
+      <c r="D4" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>lwp</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>-0.4458689170643704</v>
       </c>
-      <c r="B5" t="n">
+      <c r="C5" t="n">
         <v>32.78459680434778</v>
       </c>
-      <c r="C5" t="b">
+      <c r="D5" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ctc_annual</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>-0.8925123611712381</v>
       </c>
-      <c r="B6" t="n">
+      <c r="C6" t="n">
         <v>18.60591850893152</v>
       </c>
-      <c r="C6" t="b">
+      <c r="D6" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>gross_salary</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
         <v>-0.7487728481926048</v>
       </c>
-      <c r="B7" t="n">
+      <c r="C7" t="n">
         <v>22.69970637366298</v>
       </c>
-      <c r="C7" t="b">
+      <c r="D7" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
         <v>-0.8969096265694753</v>
       </c>
-      <c r="B8" t="n">
+      <c r="C8" t="n">
         <v>18.4883571432826</v>
       </c>
-      <c r="C8" t="b">
+      <c r="D8" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>hra</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
         <v>-0.8969037057031658</v>
       </c>
-      <c r="B9" t="n">
+      <c r="C9" t="n">
         <v>18.48851512726382</v>
       </c>
-      <c r="C9" t="b">
+      <c r="D9" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>special_allowance</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
         <v>-0.7487734683146702</v>
       </c>
-      <c r="B10" t="n">
+      <c r="C10" t="n">
         <v>22.69968768228979</v>
       </c>
-      <c r="C10" t="b">
+      <c r="D10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>conveyance</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
         <v>0.5915925417082991</v>
       </c>
-      <c r="B11" t="n">
+      <c r="C11" t="n">
         <v>72.29382653025299</v>
       </c>
-      <c r="C11" t="b">
+      <c r="D11" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>other_allowances</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
         <v>-1.324557654660229</v>
       </c>
-      <c r="B12" t="n">
+      <c r="C12" t="n">
         <v>9.265895429722764</v>
       </c>
-      <c r="C12" t="b">
+      <c r="D12" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>variable_pay</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
         <v>-0.2270710655802821</v>
       </c>
-      <c r="B13" t="n">
+      <c r="C13" t="n">
         <v>41.01842413639275</v>
       </c>
-      <c r="C13" t="b">
+      <c r="D13" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>investments_80c</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
         <v>-0.7134764738416087</v>
       </c>
-      <c r="B14" t="n">
+      <c r="C14" t="n">
         <v>23.77754830025104</v>
       </c>
-      <c r="C14" t="b">
+      <c r="D14" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>total_earnings</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
         <v>-0.7410039273935294</v>
       </c>
-      <c r="B15" t="n">
+      <c r="C15" t="n">
         <v>22.93455295125452</v>
       </c>
-      <c r="C15" t="b">
+      <c r="D15" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>pf</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
         <v>0.2589370049199478</v>
       </c>
-      <c r="B16" t="n">
+      <c r="C16" t="n">
         <v>60.21580770950496</v>
       </c>
-      <c r="C16" t="b">
+      <c r="D16" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
         <v>-0.3541441234874145</v>
       </c>
-      <c r="B17" t="n">
+      <c r="C17" t="n">
         <v>36.16154381406916</v>
       </c>
-      <c r="C17" t="b">
+      <c r="D17" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>tds</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
         <v>-0.5039287831891985</v>
       </c>
-      <c r="B18" t="n">
+      <c r="C18" t="n">
         <v>30.71557116144048</v>
       </c>
-      <c r="C18" t="b">
+      <c r="D18" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>other_deductions</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
         <v>-0.365358003149192</v>
       </c>
-      <c r="B19" t="n">
+      <c r="C19" t="n">
         <v>35.74220930849559</v>
       </c>
-      <c r="C19" t="b">
+      <c r="D19" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>total_deductions</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
         <v>-0.3748926157689837</v>
       </c>
-      <c r="B20" t="n">
+      <c r="C20" t="n">
         <v>35.38701655045149</v>
       </c>
-      <c r="C20" t="b">
+      <c r="D20" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>net_payable</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
         <v>-0.7494193580132499</v>
       </c>
-      <c r="B21" t="n">
+      <c r="C21" t="n">
         <v>22.68022434820888</v>
       </c>
-      <c r="C21" t="b">
+      <c r="D21" t="b">
         <v>0</v>
       </c>
     </row>
@@ -914,215 +1009,310 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>z_score</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>z_score_deviation (%)</t>
-        </is>
-      </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>z_score_deviation</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>anomaly</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paid_days</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>0.9078412990032004</v>
       </c>
-      <c r="B4" t="n">
+      <c r="C4" t="n">
         <v>81.80189624487603</v>
       </c>
-      <c r="C4" t="b">
+      <c r="D4" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>lwp</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>-0.4458689170643704</v>
       </c>
-      <c r="B5" t="n">
+      <c r="C5" t="n">
         <v>32.78459680434778</v>
       </c>
-      <c r="C5" t="b">
+      <c r="D5" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ctc_annual</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>-0.8925123611712381</v>
       </c>
-      <c r="B6" t="n">
+      <c r="C6" t="n">
         <v>18.60591850893152</v>
       </c>
-      <c r="C6" t="b">
+      <c r="D6" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>gross_salary</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
         <v>-0.7487728481926048</v>
       </c>
-      <c r="B7" t="n">
+      <c r="C7" t="n">
         <v>22.69970637366298</v>
       </c>
-      <c r="C7" t="b">
+      <c r="D7" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
         <v>-0.8969096265694753</v>
       </c>
-      <c r="B8" t="n">
+      <c r="C8" t="n">
         <v>18.4883571432826</v>
       </c>
-      <c r="C8" t="b">
+      <c r="D8" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>hra</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
         <v>-0.8969037057031658</v>
       </c>
-      <c r="B9" t="n">
+      <c r="C9" t="n">
         <v>18.48851512726382</v>
       </c>
-      <c r="C9" t="b">
+      <c r="D9" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>special_allowance</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
         <v>-0.7487734683146702</v>
       </c>
-      <c r="B10" t="n">
+      <c r="C10" t="n">
         <v>22.69968768228979</v>
       </c>
-      <c r="C10" t="b">
+      <c r="D10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>conveyance</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
         <v>0.5915925417082991</v>
       </c>
-      <c r="B11" t="n">
+      <c r="C11" t="n">
         <v>72.29382653025299</v>
       </c>
-      <c r="C11" t="b">
+      <c r="D11" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>other_allowances</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
         <v>-1.324557654660229</v>
       </c>
-      <c r="B12" t="n">
+      <c r="C12" t="n">
         <v>9.265895429722764</v>
       </c>
-      <c r="C12" t="b">
+      <c r="D12" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>variable_pay</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
         <v>-0.2270710655802821</v>
       </c>
-      <c r="B13" t="n">
+      <c r="C13" t="n">
         <v>41.01842413639275</v>
       </c>
-      <c r="C13" t="b">
+      <c r="D13" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>investments_80c</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
         <v>-0.7134764738416087</v>
       </c>
-      <c r="B14" t="n">
+      <c r="C14" t="n">
         <v>23.77754830025104</v>
       </c>
-      <c r="C14" t="b">
+      <c r="D14" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>total_earnings</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
         <v>-0.7410039273935294</v>
       </c>
-      <c r="B15" t="n">
+      <c r="C15" t="n">
         <v>22.93455295125452</v>
       </c>
-      <c r="C15" t="b">
+      <c r="D15" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>pf</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
         <v>0.2589370049199478</v>
       </c>
-      <c r="B16" t="n">
+      <c r="C16" t="n">
         <v>60.21580770950496</v>
       </c>
-      <c r="C16" t="b">
+      <c r="D16" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
         <v>-0.3541441234874145</v>
       </c>
-      <c r="B17" t="n">
+      <c r="C17" t="n">
         <v>36.16154381406916</v>
       </c>
-      <c r="C17" t="b">
+      <c r="D17" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>tds</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
         <v>-0.5039287831891985</v>
       </c>
-      <c r="B18" t="n">
+      <c r="C18" t="n">
         <v>30.71557116144048</v>
       </c>
-      <c r="C18" t="b">
+      <c r="D18" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>other_deductions</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
         <v>-0.365358003149192</v>
       </c>
-      <c r="B19" t="n">
+      <c r="C19" t="n">
         <v>35.74220930849559</v>
       </c>
-      <c r="C19" t="b">
+      <c r="D19" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>total_deductions</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
         <v>-0.3748926157689837</v>
       </c>
-      <c r="B20" t="n">
+      <c r="C20" t="n">
         <v>35.38701655045149</v>
       </c>
-      <c r="C20" t="b">
+      <c r="D20" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>net_payable</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
         <v>-0.7494193580132499</v>
       </c>
-      <c r="B21" t="n">
+      <c r="C21" t="n">
         <v>22.68022434820888</v>
       </c>
-      <c r="C21" t="b">
+      <c r="D21" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1400,215 +1590,310 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>z_score</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>z_score_deviation (%)</t>
-        </is>
-      </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>z_score_deviation</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>anomaly</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paid_days</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>0.9078412990032004</v>
       </c>
-      <c r="B4" t="n">
+      <c r="C4" t="n">
         <v>81.80189624487603</v>
       </c>
-      <c r="C4" t="b">
+      <c r="D4" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>lwp</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>-0.4458689170643704</v>
       </c>
-      <c r="B5" t="n">
+      <c r="C5" t="n">
         <v>32.78459680434778</v>
       </c>
-      <c r="C5" t="b">
+      <c r="D5" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ctc_annual</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>-0.8925123611712381</v>
       </c>
-      <c r="B6" t="n">
+      <c r="C6" t="n">
         <v>18.60591850893152</v>
       </c>
-      <c r="C6" t="b">
+      <c r="D6" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>gross_salary</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
         <v>-0.7487728481926048</v>
       </c>
-      <c r="B7" t="n">
+      <c r="C7" t="n">
         <v>22.69970637366298</v>
       </c>
-      <c r="C7" t="b">
+      <c r="D7" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
         <v>-0.8969096265694753</v>
       </c>
-      <c r="B8" t="n">
+      <c r="C8" t="n">
         <v>18.4883571432826</v>
       </c>
-      <c r="C8" t="b">
+      <c r="D8" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>hra</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
         <v>-0.8969037057031658</v>
       </c>
-      <c r="B9" t="n">
+      <c r="C9" t="n">
         <v>18.48851512726382</v>
       </c>
-      <c r="C9" t="b">
+      <c r="D9" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>special_allowance</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
         <v>-0.7487734683146702</v>
       </c>
-      <c r="B10" t="n">
+      <c r="C10" t="n">
         <v>22.69968768228979</v>
       </c>
-      <c r="C10" t="b">
+      <c r="D10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>conveyance</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
         <v>0.5915925417082991</v>
       </c>
-      <c r="B11" t="n">
+      <c r="C11" t="n">
         <v>72.29382653025299</v>
       </c>
-      <c r="C11" t="b">
+      <c r="D11" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>other_allowances</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
         <v>-1.324557654660229</v>
       </c>
-      <c r="B12" t="n">
+      <c r="C12" t="n">
         <v>9.265895429722764</v>
       </c>
-      <c r="C12" t="b">
+      <c r="D12" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>variable_pay</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
         <v>-0.2270710655802821</v>
       </c>
-      <c r="B13" t="n">
+      <c r="C13" t="n">
         <v>41.01842413639275</v>
       </c>
-      <c r="C13" t="b">
+      <c r="D13" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>investments_80c</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
         <v>-0.7134764738416087</v>
       </c>
-      <c r="B14" t="n">
+      <c r="C14" t="n">
         <v>23.77754830025104</v>
       </c>
-      <c r="C14" t="b">
+      <c r="D14" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>total_earnings</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
         <v>-0.7410039273935294</v>
       </c>
-      <c r="B15" t="n">
+      <c r="C15" t="n">
         <v>22.93455295125452</v>
       </c>
-      <c r="C15" t="b">
+      <c r="D15" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>pf</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
         <v>0.2589370049199478</v>
       </c>
-      <c r="B16" t="n">
+      <c r="C16" t="n">
         <v>60.21580770950496</v>
       </c>
-      <c r="C16" t="b">
+      <c r="D16" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
         <v>-0.3541441234874145</v>
       </c>
-      <c r="B17" t="n">
+      <c r="C17" t="n">
         <v>36.16154381406916</v>
       </c>
-      <c r="C17" t="b">
+      <c r="D17" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>tds</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
         <v>-0.5039287831891985</v>
       </c>
-      <c r="B18" t="n">
+      <c r="C18" t="n">
         <v>30.71557116144048</v>
       </c>
-      <c r="C18" t="b">
+      <c r="D18" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>other_deductions</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
         <v>-0.365358003149192</v>
       </c>
-      <c r="B19" t="n">
+      <c r="C19" t="n">
         <v>35.74220930849559</v>
       </c>
-      <c r="C19" t="b">
+      <c r="D19" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>total_deductions</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
         <v>-0.3748926157689837</v>
       </c>
-      <c r="B20" t="n">
+      <c r="C20" t="n">
         <v>35.38701655045149</v>
       </c>
-      <c r="C20" t="b">
+      <c r="D20" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>net_payable</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
         <v>-0.7494193580132499</v>
       </c>
-      <c r="B21" t="n">
+      <c r="C21" t="n">
         <v>22.68022434820888</v>
       </c>
-      <c r="C21" t="b">
+      <c r="D21" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added data exportation via database system
</commit_message>
<xml_diff>
--- a/data/output/output_data.xlsx
+++ b/data/output/output_data.xlsx
@@ -787,10 +787,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.5000066733400067</v>
+        <v>0.5</v>
       </c>
       <c r="C27" t="n">
-        <v>4.117726550623146e-06</v>
+        <v>0</v>
       </c>
       <c r="D27" t="b">
         <v>0</v>
@@ -1368,10 +1368,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.5000066733400067</v>
+        <v>0.5</v>
       </c>
       <c r="C27" t="n">
-        <v>4.117726550623146e-06</v>
+        <v>0</v>
       </c>
       <c r="D27" t="b">
         <v>0</v>
@@ -1949,10 +1949,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.5000066733400067</v>
+        <v>0.5</v>
       </c>
       <c r="C27" t="n">
-        <v>4.117726550623146e-06</v>
+        <v>0</v>
       </c>
       <c r="D27" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
added download excel file functionality; backend endpoint & frontend
</commit_message>
<xml_diff>
--- a/data/output/output_data.xlsx
+++ b/data/output/output_data.xlsx
@@ -981,7 +981,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>No Anomaly</t>
+          <t>Anomaly</t>
         </is>
       </c>
     </row>
@@ -1562,7 +1562,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>No Anomaly</t>
+          <t>Anomaly</t>
         </is>
       </c>
     </row>
@@ -2143,7 +2143,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>No Anomaly</t>
+          <t>Anomaly</t>
         </is>
       </c>
     </row>

</xml_diff>